<commit_message>
Added code to generate 1 million random samples from the 100 Monte Carlo realizations for each basin generated using the Rutherford et al. model.
</commit_message>
<xml_diff>
--- a/Other input data/Key sim results 20230830.xlsx
+++ b/Other input data/Key sim results 20230830.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/evansherwin/PycharmProjects/MethaneDistributionsPublished/Other input data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D6A7AFB-EA0B-E04A-B327-EDBEF87F570E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12F1CC56-2705-D141-89D1-810E0E639D44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9680" yWindow="460" windowWidth="29900" windowHeight="18520" activeTab="2" xr2:uid="{DA729304-F74A-A044-AD1E-035DDE35C875}"/>
+    <workbookView xWindow="9680" yWindow="460" windowWidth="29900" windowHeight="18520" xr2:uid="{DA729304-F74A-A044-AD1E-035DDE35C875}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="9" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="407">
   <si>
     <t>Kairos Permian</t>
   </si>
@@ -608,9 +608,6 @@
     <t>Logormal fit mean</t>
   </si>
   <si>
-    <t>From Jupyter code</t>
-  </si>
-  <si>
     <t>Lognormal/This study</t>
   </si>
   <si>
@@ -1263,6 +1260,27 @@
   </si>
   <si>
     <t>Table 22</t>
+  </si>
+  <si>
+    <t>From DistributionsMain.ipynb</t>
+  </si>
+  <si>
+    <t>Table 18</t>
+  </si>
+  <si>
+    <t># emissions detected</t>
+  </si>
+  <si>
+    <t>Avg. visits/site</t>
+  </si>
+  <si>
+    <t>Avg. % sites emitting</t>
+  </si>
+  <si>
+    <t># sources detected</t>
+  </si>
+  <si>
+    <t>Avg. instantaneous sources</t>
   </si>
 </sst>
 </file>
@@ -1689,707 +1707,707 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
@@ -2397,7 +2415,7 @@
         <v>57</v>
       </c>
       <c r="B142" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -2454,40 +2472,40 @@
         <v>89</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>232</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>52</v>
@@ -2505,13 +2523,13 @@
         <v>55</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>234</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>235</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>12</v>
@@ -2556,7 +2574,7 @@
         <v>48</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AK1" s="1" t="s">
         <v>16</v>
@@ -2571,7 +2589,7 @@
         <v>119</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AP1" s="1" t="s">
         <v>40</v>
@@ -2589,40 +2607,40 @@
         <v>121</v>
       </c>
       <c r="AU1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="AV1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="BF1" s="1" t="s">
-        <v>248</v>
       </c>
       <c r="BG1" s="1" t="s">
         <v>68</v>
@@ -2733,13 +2751,13 @@
         <v>143</v>
       </c>
       <c r="CQ1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="CR1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="CR1" s="1" t="s">
+      <c r="CS1" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="CS1" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="CT1" s="1" t="s">
         <v>144</v>
@@ -2841,22 +2859,22 @@
         <v>180</v>
       </c>
       <c r="EA1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="EB1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="EB1" s="1" t="s">
+      <c r="EC1" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="EC1" s="1" t="s">
+      <c r="ED1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="ED1" s="1" t="s">
+      <c r="EE1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="EE1" s="1" t="s">
+      <c r="EF1" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="EF1" s="1" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:136" x14ac:dyDescent="0.2">
@@ -10880,6 +10898,10 @@
       <c r="CA23" s="12"/>
       <c r="CB23" s="12"/>
       <c r="CC23" s="12"/>
+      <c r="CD23" s="10">
+        <f>CD3+CD7+CD13+CD14+CD15+CD16</f>
+        <v>104249</v>
+      </c>
       <c r="CH23" s="10">
         <f>CH3+CH7+CH13+CH14+CH15+CH16</f>
         <v>527.06480186705596</v>
@@ -11092,7 +11114,7 @@
         <v>8760</v>
       </c>
       <c r="Y27" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AA27" s="10">
         <f>SUM(W2:W6)</f>
@@ -11702,6 +11724,8 @@
     <col min="1" max="1" width="24.1640625" customWidth="1"/>
     <col min="2" max="2" width="14.1640625" customWidth="1"/>
     <col min="8" max="8" width="16.33203125" customWidth="1"/>
+    <col min="10" max="10" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
     <col min="23" max="23" width="13.1640625" customWidth="1"/>
     <col min="27" max="27" width="18.83203125" customWidth="1"/>
@@ -11709,12 +11733,12 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="J1" t="s">
-        <v>182</v>
+        <v>400</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="22" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B2" t="str" cm="1">
         <f t="array" ref="B2:B21">'By site'!Y1:Y20</f>
@@ -11733,7 +11757,7 @@
         <v># production plumes sel</v>
       </c>
       <c r="H2" s="22" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I2" t="s">
         <v>156</v>
@@ -11742,10 +11766,10 @@
         <v>181</v>
       </c>
       <c r="K2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="M2" s="22" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="N2" t="str" cm="1">
         <f t="array" ref="N2:N21">'By site'!CD1:CD20</f>
@@ -11796,11 +11820,11 @@
         <v>6.052388365933389</v>
       </c>
       <c r="J3" s="11">
-        <v>3.1618550000000001</v>
+        <v>3.1778710000000001</v>
       </c>
       <c r="K3" s="9">
         <f>J3/I3</f>
-        <v>0.52241442697181972</v>
+        <v>0.52506065504438504</v>
       </c>
       <c r="M3" t="s">
         <v>90</v>
@@ -11848,11 +11872,11 @@
         <v>6.606866938276907</v>
       </c>
       <c r="J4" s="11">
-        <v>3.8726229999999999</v>
+        <v>3.850206</v>
       </c>
       <c r="K4" s="9">
         <f t="shared" ref="K4:K17" si="0">J4/I4</f>
-        <v>0.5861512024048714</v>
+        <v>0.58275821746822509</v>
       </c>
       <c r="M4" t="s">
         <v>73</v>
@@ -11900,11 +11924,11 @@
         <v>6.1276230429662357</v>
       </c>
       <c r="J5" s="11">
-        <v>5.3088649999999999</v>
+        <v>5.3650339999999996</v>
       </c>
       <c r="K5" s="9">
         <f t="shared" si="0"/>
-        <v>0.86638243945079652</v>
+        <v>0.87554896284920869</v>
       </c>
       <c r="M5" t="s">
         <v>74</v>
@@ -11952,11 +11976,11 @@
         <v>6.2349792015267536</v>
       </c>
       <c r="J6" s="11">
-        <v>7.6787859999999997</v>
+        <v>7.7054330000000002</v>
       </c>
       <c r="K6" s="9">
         <f t="shared" si="0"/>
-        <v>1.2315656158275079</v>
+        <v>1.2358394071488126</v>
       </c>
       <c r="M6" t="s">
         <v>76</v>
@@ -12004,11 +12028,11 @@
         <v>6.0949560498492064</v>
       </c>
       <c r="J7" s="11">
-        <v>7.5557819999999998</v>
+        <v>7.5237049999999996</v>
       </c>
       <c r="K7" s="9">
         <f t="shared" si="0"/>
-        <v>1.2396778480768431</v>
+        <v>1.2344149717348891</v>
       </c>
       <c r="M7" t="s">
         <v>75</v>
@@ -12056,11 +12080,11 @@
         <v>0.18945091670818651</v>
       </c>
       <c r="J8" s="11">
-        <v>0.522096</v>
+        <v>0.51518399999999998</v>
       </c>
       <c r="K8" s="9">
         <f t="shared" si="0"/>
-        <v>2.7558378131481445</v>
+        <v>2.7193534291182342</v>
       </c>
       <c r="M8" t="s">
         <v>77</v>
@@ -12108,11 +12132,11 @@
         <v>0.27423144190568932</v>
       </c>
       <c r="J9" s="11">
-        <v>0.54015999999999997</v>
+        <v>0.50656199999999996</v>
       </c>
       <c r="K9" s="9">
         <f t="shared" si="0"/>
-        <v>1.9697230786022191</v>
+        <v>1.8472061280785272</v>
       </c>
       <c r="M9" t="s">
         <v>78</v>
@@ -12160,11 +12184,11 @@
         <v>0.35380735175756123</v>
       </c>
       <c r="J10" s="11">
-        <v>0.54778199999999999</v>
+        <v>0.54781199999999997</v>
       </c>
       <c r="K10" s="9">
         <f t="shared" si="0"/>
-        <v>1.5482493432622499</v>
+        <v>1.5483341351690629</v>
       </c>
       <c r="M10" t="s">
         <v>80</v>
@@ -12212,11 +12236,11 @@
         <v>0.27576139902140961</v>
       </c>
       <c r="J11" s="11">
-        <v>0.54308299999999998</v>
+        <v>0.54293000000000002</v>
       </c>
       <c r="K11" s="9">
         <f t="shared" si="0"/>
-        <v>1.9693945632972221</v>
+        <v>1.9688397358248386</v>
       </c>
       <c r="M11" t="s">
         <v>79</v>
@@ -12264,11 +12288,11 @@
         <v>0.20820187602300366</v>
       </c>
       <c r="J12" s="11">
-        <v>0.51156699999999999</v>
+        <v>0.51121399999999995</v>
       </c>
       <c r="K12" s="9">
         <f t="shared" si="0"/>
-        <v>2.4570720003669821</v>
+        <v>2.4553765305338424</v>
       </c>
       <c r="M12" t="s">
         <v>81</v>
@@ -12316,11 +12340,11 @@
         <v>2.0054687273338159</v>
       </c>
       <c r="J13" s="11">
-        <v>4.5976879999999998</v>
+        <v>4.6079460000000001</v>
       </c>
       <c r="K13" s="9">
         <f t="shared" si="0"/>
-        <v>2.2925752654903913</v>
+        <v>2.2976902791827949</v>
       </c>
       <c r="M13" t="s">
         <v>82</v>
@@ -12368,11 +12392,11 @@
         <v>2.0146506103738195</v>
       </c>
       <c r="J14" s="11">
-        <v>4.5944459999999996</v>
+        <v>4.6101710000000002</v>
       </c>
       <c r="K14" s="9">
         <f t="shared" si="0"/>
-        <v>2.2805175132314868</v>
+        <v>2.2883228368538702</v>
       </c>
       <c r="M14" t="s">
         <v>83</v>
@@ -12420,11 +12444,11 @@
         <v>3.9334964797278733</v>
       </c>
       <c r="J15" s="11">
-        <v>1.664976</v>
+        <v>1.671362</v>
       </c>
       <c r="K15" s="9">
         <f t="shared" si="0"/>
-        <v>0.42328142622748355</v>
+        <v>0.42490491821048432</v>
       </c>
       <c r="M15" t="s">
         <v>84</v>
@@ -12472,11 +12496,11 @@
         <v>3.0595424391411652</v>
       </c>
       <c r="J16" s="11">
-        <v>3.5822560000000001</v>
+        <v>3.5833330000000001</v>
       </c>
       <c r="K16" s="9">
         <f t="shared" si="0"/>
-        <v>1.1708469718124139</v>
+        <v>1.1711989852331863</v>
       </c>
       <c r="M16" t="s">
         <v>72</v>
@@ -12524,11 +12548,11 @@
         <v>3.3027910836604355</v>
       </c>
       <c r="J17" s="11">
-        <v>1.631947</v>
+        <v>1.565739</v>
       </c>
       <c r="K17" s="9">
         <f t="shared" si="0"/>
-        <v>0.49411148288293694</v>
+        <v>0.47406540720847357</v>
       </c>
       <c r="M17" t="s">
         <v>85</v>
@@ -12762,7 +12786,7 @@
         <v>160</v>
       </c>
       <c r="G24" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="H24" t="s">
         <v>164</v>
@@ -12777,7 +12801,7 @@
         <v>167</v>
       </c>
       <c r="N24" s="22" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="O24" t="s">
         <v>168</v>
@@ -12792,7 +12816,7 @@
         <v>171</v>
       </c>
       <c r="T24" s="22" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="U24" t="s">
         <v>172</v>
@@ -14279,34 +14303,34 @@
         <v>157</v>
       </c>
       <c r="B47" t="s">
+        <v>183</v>
+      </c>
+      <c r="C47" t="s">
         <v>184</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>185</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>186</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>187</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>188</v>
-      </c>
-      <c r="G47" t="s">
-        <v>189</v>
       </c>
       <c r="I47" s="22" t="s">
         <v>158</v>
       </c>
       <c r="J47" t="s">
+        <v>189</v>
+      </c>
+      <c r="K47" t="s">
         <v>190</v>
       </c>
-      <c r="K47" t="s">
+      <c r="L47" t="s">
         <v>191</v>
-      </c>
-      <c r="L47" t="s">
-        <v>192</v>
       </c>
       <c r="O47" s="22" t="s">
         <v>163</v>
@@ -14320,22 +14344,22 @@
         <v>SErr of sample mean</v>
       </c>
       <c r="T47" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="U47" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Y47" s="22" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="Z47" t="s">
+        <v>207</v>
+      </c>
+      <c r="AA47" t="s">
+        <v>206</v>
+      </c>
+      <c r="AB47" t="s">
         <v>208</v>
-      </c>
-      <c r="AA47" t="s">
-        <v>207</v>
-      </c>
-      <c r="AB47" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="48" spans="1:28" x14ac:dyDescent="0.2">
@@ -15923,7 +15947,7 @@
         <v>0.76974677953887372</v>
       </c>
       <c r="Y67" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="Z67">
         <v>20.9</v>
@@ -15938,79 +15962,106 @@
         <v>0.89820657805016646</v>
       </c>
     </row>
-    <row r="68" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A68" s="22" t="s">
-        <v>391</v>
-      </c>
-      <c r="B68" t="s">
-        <v>216</v>
-      </c>
-      <c r="C68" t="s">
+    <row r="69" spans="1:28" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="22" t="s">
         <v>390</v>
       </c>
-      <c r="D68" t="s">
-        <v>388</v>
-      </c>
-      <c r="E68" t="s">
+      <c r="B69" t="s">
+        <v>215</v>
+      </c>
+      <c r="C69" t="s">
+        <v>389</v>
+      </c>
+      <c r="D69" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="69" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+      <c r="E69" t="s">
+        <v>386</v>
+      </c>
+      <c r="I69" s="22" t="s">
+        <v>401</v>
+      </c>
+      <c r="J69" t="s">
+        <v>136</v>
+      </c>
+      <c r="K69" t="s">
+        <v>402</v>
+      </c>
+      <c r="L69" t="s">
+        <v>405</v>
+      </c>
+      <c r="M69" t="s">
+        <v>403</v>
+      </c>
+      <c r="N69" t="s">
+        <v>406</v>
+      </c>
+      <c r="O69" t="s">
+        <v>404</v>
+      </c>
+      <c r="Z69" t="s">
+        <v>213</v>
+      </c>
+      <c r="AA69" t="s">
+        <v>210</v>
+      </c>
+      <c r="AB69" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="70" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>90</v>
       </c>
-      <c r="B69">
+      <c r="B70">
         <f>'By site'!DN2*'By site'!Z2</f>
         <v>24.357965236152825</v>
       </c>
-      <c r="C69" s="5">
+      <c r="C70" s="5">
         <f>'By site'!DX2</f>
         <v>7.2701047721023199E-3</v>
       </c>
-      <c r="D69" s="2">
-        <f>'By site'!DU2/C69-1</f>
+      <c r="D70" s="2">
+        <f>'By site'!DU2/C70-1</f>
         <v>0.65124376861340028</v>
       </c>
-      <c r="E69" t="b">
-        <f>ABS(D69) &lt;= 0.5</f>
-        <v>0</v>
-      </c>
-      <c r="F69">
-        <f>COUNTIF(E69:E83, TRUE)</f>
+      <c r="E70" t="b">
+        <f>ABS(D70) &lt;= 0.5</f>
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <f>COUNTIF(E70:E84, TRUE)</f>
         <v>7</v>
       </c>
-      <c r="Z69" t="s">
-        <v>214</v>
-      </c>
-      <c r="AA69" t="s">
-        <v>211</v>
-      </c>
-      <c r="AB69" t="s">
+      <c r="I70" t="s">
+        <v>90</v>
+      </c>
+      <c r="J70" s="7">
+        <f>'By site'!CD2</f>
+        <v>18030</v>
+      </c>
+      <c r="K70" s="7">
+        <f>'By site'!AD2</f>
+        <v>1279</v>
+      </c>
+      <c r="L70">
+        <f>'By site'!AF2</f>
+        <v>627</v>
+      </c>
+      <c r="M70" s="6">
+        <f>'By site'!AQ2</f>
+        <v>3.76982806433722</v>
+      </c>
+      <c r="N70" s="6">
+        <f>'By site'!AG2</f>
+        <v>299.73599999999999</v>
+      </c>
+      <c r="O70" s="5">
+        <f>'By site'!CG2</f>
+        <v>1.6624292845257901E-2</v>
+      </c>
+      <c r="Y70" t="s">
         <v>212</v>
-      </c>
-    </row>
-    <row r="70" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>73</v>
-      </c>
-      <c r="B70">
-        <f>'By site'!DN3*'By site'!Z3</f>
-        <v>120.97259424653235</v>
-      </c>
-      <c r="C70" s="5">
-        <f>'By site'!DX3</f>
-        <v>6.5124999847487302E-3</v>
-      </c>
-      <c r="D70" s="2">
-        <f>'By site'!DU3/C70-1</f>
-        <v>0.22683425264099366</v>
-      </c>
-      <c r="E70" t="b">
-        <f t="shared" ref="E70:E87" si="2">ABS(D70) &lt;= 0.5</f>
-        <v>1</v>
-      </c>
-      <c r="Y70" t="s">
-        <v>213</v>
       </c>
       <c r="Z70">
         <f>'By site'!CQ14 - 'By site'!CQ20</f>
@@ -16027,398 +16078,814 @@
     </row>
     <row r="71" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71">
+        <f>'By site'!DN3*'By site'!Z3</f>
+        <v>120.97259424653235</v>
+      </c>
+      <c r="C71" s="5">
+        <f>'By site'!DX3</f>
+        <v>6.5124999847487302E-3</v>
+      </c>
+      <c r="D71" s="2">
+        <f>'By site'!DU3/C71-1</f>
+        <v>0.22683425264099366</v>
+      </c>
+      <c r="E71" t="b">
+        <f t="shared" ref="E71:E88" si="2">ABS(D71) &lt;= 0.5</f>
+        <v>1</v>
+      </c>
+      <c r="I71" t="s">
+        <v>73</v>
+      </c>
+      <c r="J71" s="7">
+        <f>'By site'!CD3</f>
+        <v>46337</v>
+      </c>
+      <c r="K71" s="7">
+        <f>'By site'!AD3</f>
+        <v>1749</v>
+      </c>
+      <c r="L71">
+        <f>'By site'!AF3</f>
+        <v>1054</v>
+      </c>
+      <c r="M71" s="6">
+        <f>'By site'!AQ3</f>
+        <v>3.8655933703088201</v>
+      </c>
+      <c r="N71" s="6">
+        <f>'By site'!AG3</f>
+        <v>483.46499999999997</v>
+      </c>
+      <c r="O71" s="5">
+        <f>'By site'!CG3</f>
+        <v>1.04336707167059E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
         <v>74</v>
       </c>
-      <c r="B71">
+      <c r="B72">
         <f>'By site'!DN4*'By site'!Z4</f>
         <v>50.816506638195825</v>
       </c>
-      <c r="C71" s="5">
+      <c r="C72" s="5">
         <f>'By site'!DX4</f>
         <v>5.9587925946185498E-3</v>
       </c>
-      <c r="D71" s="2">
-        <f>'By site'!DU4/C71-1</f>
+      <c r="D72" s="2">
+        <f>'By site'!DU4/C72-1</f>
         <v>-4.7912009924108712E-2</v>
-      </c>
-      <c r="E71" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>76</v>
-      </c>
-      <c r="B72">
-        <f>'By site'!DN5*'By site'!Z5</f>
-        <v>63.438241032096158</v>
-      </c>
-      <c r="C72" s="5">
-        <f>'By site'!DX5</f>
-        <v>5.9587925946185498E-3</v>
-      </c>
-      <c r="D72" s="2">
-        <f>'By site'!DU5/C72-1</f>
-        <v>-1.4352765550062596E-2</v>
       </c>
       <c r="E72" t="b">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
+      <c r="I72" t="s">
+        <v>74</v>
+      </c>
+      <c r="J72" s="7">
+        <f>'By site'!CD4</f>
+        <v>9380</v>
+      </c>
+      <c r="K72" s="7">
+        <f>'By site'!AD4</f>
+        <v>284</v>
+      </c>
+      <c r="L72">
+        <f>'By site'!AF4</f>
+        <v>239</v>
+      </c>
+      <c r="M72" s="6">
+        <f>'By site'!AQ4</f>
+        <v>2.85575692963753</v>
+      </c>
+      <c r="N72" s="6">
+        <f>'By site'!AG4</f>
+        <v>101.235</v>
+      </c>
+      <c r="O72" s="5">
+        <f>'By site'!CG4</f>
+        <v>1.07926439232409E-2</v>
+      </c>
     </row>
     <row r="73" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B73">
-        <f>'By site'!DN6*'By site'!Z6</f>
-        <v>66.395754134398558</v>
+        <f>'By site'!DN5*'By site'!Z5</f>
+        <v>63.438241032096158</v>
       </c>
       <c r="C73" s="5">
-        <f>'By site'!DX6</f>
+        <f>'By site'!DX5</f>
         <v>5.9587925946185498E-3</v>
       </c>
       <c r="D73" s="2">
-        <f>'By site'!DU6/C73-1</f>
-        <v>-9.393662715129758E-3</v>
+        <f>'By site'!DU5/C73-1</f>
+        <v>-1.4352765550062596E-2</v>
       </c>
       <c r="E73" t="b">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
+      <c r="I73" t="s">
+        <v>76</v>
+      </c>
+      <c r="J73" s="7">
+        <f>'By site'!CD5</f>
+        <v>10432</v>
+      </c>
+      <c r="K73" s="7">
+        <f>'By site'!AD5</f>
+        <v>416</v>
+      </c>
+      <c r="L73">
+        <f>'By site'!AF5</f>
+        <v>296</v>
+      </c>
+      <c r="M73" s="6">
+        <f>'By site'!AQ5</f>
+        <v>4.82716641104295</v>
+      </c>
+      <c r="N73" s="6">
+        <f>'By site'!AG5</f>
+        <v>124.633</v>
+      </c>
+      <c r="O73" s="5">
+        <f>'By site'!CG5</f>
+        <v>1.1947181748466301E-2</v>
+      </c>
     </row>
     <row r="74" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
+        <v>75</v>
+      </c>
+      <c r="B74">
+        <f>'By site'!DN6*'By site'!Z6</f>
+        <v>66.395754134398558</v>
+      </c>
+      <c r="C74" s="5">
+        <f>'By site'!DX6</f>
+        <v>5.9587925946185498E-3</v>
+      </c>
+      <c r="D74" s="2">
+        <f>'By site'!DU6/C74-1</f>
+        <v>-9.393662715129758E-3</v>
+      </c>
+      <c r="E74" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="I74" t="s">
+        <v>75</v>
+      </c>
+      <c r="J74" s="7">
+        <f>'By site'!CD6</f>
+        <v>10777</v>
+      </c>
+      <c r="K74" s="7">
+        <f>'By site'!AD6</f>
+        <v>334</v>
+      </c>
+      <c r="L74">
+        <f>'By site'!AF6</f>
+        <v>232</v>
+      </c>
+      <c r="M74" s="6">
+        <f>'By site'!AQ6</f>
+        <v>4.7946552844019701</v>
+      </c>
+      <c r="N74" s="6">
+        <f>'By site'!AG6</f>
+        <v>92.781000000000006</v>
+      </c>
+      <c r="O74" s="5">
+        <f>'By site'!CG6</f>
+        <v>8.6091676718938505E-3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
         <v>77</v>
       </c>
-      <c r="B74">
+      <c r="B75">
         <f>'By site'!DN7*'By site'!Z7</f>
         <v>15.196735288855514</v>
       </c>
-      <c r="C74" s="5">
+      <c r="C75" s="5">
         <f>'By site'!DX7</f>
         <v>5.1203661661178103E-2</v>
       </c>
-      <c r="D74" s="2">
-        <f>'By site'!DU7/C74-1</f>
+      <c r="D75" s="2">
+        <f>'By site'!DU7/C75-1</f>
         <v>-0.78594640514429326</v>
       </c>
-      <c r="E74" t="b">
+      <c r="E75" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
+      <c r="I75" t="s">
+        <v>77</v>
+      </c>
+      <c r="J75" s="7">
+        <f>'By site'!CD7</f>
+        <v>27698</v>
+      </c>
+      <c r="K75" s="7">
+        <f>'By site'!AD7</f>
+        <v>77</v>
+      </c>
+      <c r="L75">
+        <f>'By site'!AF7</f>
+        <v>40</v>
+      </c>
+      <c r="M75" s="6">
+        <f>'By site'!AQ7</f>
+        <v>1.9552314246516</v>
+      </c>
+      <c r="N75" s="6">
+        <f>'By site'!AG7</f>
+        <v>15.076000000000001</v>
+      </c>
+      <c r="O75" s="5">
+        <f>'By site'!CG7</f>
+        <v>5.4429922738103798E-4</v>
+      </c>
+    </row>
+    <row r="76" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
         <v>78</v>
       </c>
-      <c r="B75">
+      <c r="B76">
         <f>'By site'!DN8*'By site'!Z8</f>
         <v>15.50160821102906</v>
       </c>
-      <c r="C75" s="5">
+      <c r="C76" s="5">
         <f>'By site'!DX8</f>
         <v>4.8477730768718801E-2</v>
       </c>
-      <c r="D75" s="2">
-        <f>'By site'!DU8/C75-1</f>
+      <c r="D76" s="2">
+        <f>'By site'!DU8/C76-1</f>
         <v>-0.78799691204898947</v>
       </c>
-      <c r="E75" t="b">
+      <c r="E76" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
+      <c r="I76" t="s">
+        <v>78</v>
+      </c>
+      <c r="J76" s="7">
+        <f>'By site'!CD8</f>
+        <v>26910</v>
+      </c>
+      <c r="K76" s="7">
+        <f>'By site'!AD8</f>
+        <v>86</v>
+      </c>
+      <c r="L76">
+        <f>'By site'!AF8</f>
+        <v>54</v>
+      </c>
+      <c r="M76" s="6">
+        <f>'By site'!AQ8</f>
+        <v>4.7679672984020796</v>
+      </c>
+      <c r="N76" s="6">
+        <f>'By site'!AG8</f>
+        <v>15.933</v>
+      </c>
+      <c r="O76" s="5">
+        <f>'By site'!CG8</f>
+        <v>5.9208472686733595E-4</v>
+      </c>
+    </row>
+    <row r="77" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
         <v>80</v>
       </c>
-      <c r="B76">
+      <c r="B77">
         <f>'By site'!DN9*'By site'!Z9</f>
         <v>14.261429630091026</v>
       </c>
-      <c r="C76" s="5">
+      <c r="C77" s="5">
         <f>'By site'!DX9</f>
         <v>5.6475808579374398E-2</v>
       </c>
-      <c r="D76" s="2">
-        <f>'By site'!DU9/C76-1</f>
+      <c r="D77" s="2">
+        <f>'By site'!DU9/C77-1</f>
         <v>-0.8582157338196954</v>
       </c>
-      <c r="E76" t="b">
+      <c r="E77" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
+      <c r="I77" t="s">
+        <v>80</v>
+      </c>
+      <c r="J77" s="7">
+        <f>'By site'!CD9</f>
+        <v>15992</v>
+      </c>
+      <c r="K77" s="7">
+        <f>'By site'!AD9</f>
+        <v>94</v>
+      </c>
+      <c r="L77">
+        <f>'By site'!AF9</f>
+        <v>39</v>
+      </c>
+      <c r="M77" s="6">
+        <f>'By site'!AQ9</f>
+        <v>7.4688594297148603</v>
+      </c>
+      <c r="N77" s="6">
+        <f>'By site'!AG9</f>
+        <v>13.333</v>
+      </c>
+      <c r="O77" s="5">
+        <f>'By site'!CG9</f>
+        <v>8.3372936468234103E-4</v>
+      </c>
+    </row>
+    <row r="78" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
         <v>79</v>
       </c>
-      <c r="B77">
+      <c r="B78">
         <f>'By site'!DN10*'By site'!Z10</f>
         <v>15.112625086571196</v>
       </c>
-      <c r="C77" s="5">
+      <c r="C78" s="5">
         <f>'By site'!DX10</f>
         <v>5.6475808579374398E-2</v>
       </c>
-      <c r="D77" s="2">
-        <f>'By site'!DU10/C77-1</f>
+      <c r="D78" s="2">
+        <f>'By site'!DU10/C78-1</f>
         <v>-0.85391334038433309</v>
       </c>
-      <c r="E77" t="b">
+      <c r="E78" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
+      <c r="I78" t="s">
+        <v>79</v>
+      </c>
+      <c r="J78" s="7">
+        <f>'By site'!CD10</f>
+        <v>16579</v>
+      </c>
+      <c r="K78" s="7">
+        <f>'By site'!AD10</f>
+        <v>48</v>
+      </c>
+      <c r="L78">
+        <f>'By site'!AF10</f>
+        <v>27</v>
+      </c>
+      <c r="M78" s="6">
+        <f>'By site'!AQ10</f>
+        <v>7.2219675493093698</v>
+      </c>
+      <c r="N78" s="6">
+        <f>'By site'!AG10</f>
+        <v>8.0850000000000009</v>
+      </c>
+      <c r="O78" s="5">
+        <f>'By site'!CG10</f>
+        <v>4.8766511852343301E-4</v>
+      </c>
+    </row>
+    <row r="79" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
         <v>81</v>
       </c>
-      <c r="B78">
+      <c r="B79">
         <f>'By site'!DN11*'By site'!Z11</f>
         <v>12.20299091396601</v>
       </c>
-      <c r="C78" s="5">
+      <c r="C79" s="5">
         <f>'By site'!DX11</f>
         <v>5.6475808579374398E-2</v>
       </c>
-      <c r="D78" s="2">
-        <f>'By site'!DU11/C78-1</f>
+      <c r="D79" s="2">
+        <f>'By site'!DU11/C79-1</f>
         <v>-0.838365354689527</v>
       </c>
-      <c r="E78" t="b">
+      <c r="E79" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
+      <c r="I79" t="s">
+        <v>81</v>
+      </c>
+      <c r="J79" s="7">
+        <f>'By site'!CD11</f>
+        <v>16743</v>
+      </c>
+      <c r="K79" s="7">
+        <f>'By site'!AD11</f>
+        <v>47</v>
+      </c>
+      <c r="L79">
+        <f>'By site'!AF11</f>
+        <v>35</v>
+      </c>
+      <c r="M79" s="6">
+        <f>'By site'!AQ11</f>
+        <v>3.5712237950188102</v>
+      </c>
+      <c r="N79" s="6">
+        <f>'By site'!AG11</f>
+        <v>15.747999999999999</v>
+      </c>
+      <c r="O79" s="5">
+        <f>'By site'!CG11</f>
+        <v>9.4057217941826397E-4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
         <v>82</v>
       </c>
-      <c r="B79">
+      <c r="B80">
         <f>'By site'!DN12*'By site'!Z12</f>
         <v>19.391289447219531</v>
       </c>
-      <c r="C79" s="5">
+      <c r="C80" s="5">
         <f>'By site'!DX12</f>
         <v>5.4262313508968698E-3</v>
       </c>
-      <c r="D79" s="2">
-        <f>'By site'!DU12/C79-1</f>
+      <c r="D80" s="2">
+        <f>'By site'!DU12/C80-1</f>
         <v>0.15804321203166483</v>
-      </c>
-      <c r="E79" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
-        <v>83</v>
-      </c>
-      <c r="B80">
-        <f>'By site'!DN13*'By site'!Z13</f>
-        <v>19.151798216419305</v>
-      </c>
-      <c r="C80" s="5">
-        <f>'By site'!DX13</f>
-        <v>5.4262313508968698E-3</v>
-      </c>
-      <c r="D80" s="2">
-        <f>'By site'!DU13/C80-1</f>
-        <v>0.1819075310481173</v>
       </c>
       <c r="E80" t="b">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="I80" t="s">
+        <v>82</v>
+      </c>
+      <c r="J80" s="7">
+        <f>'By site'!CD12</f>
+        <v>7254</v>
+      </c>
+      <c r="K80" s="7">
+        <f>'By site'!AD12</f>
+        <v>34</v>
+      </c>
+      <c r="L80">
+        <f>'By site'!AF12</f>
+        <v>27</v>
+      </c>
+      <c r="M80" s="6">
+        <f>'By site'!AQ12</f>
+        <v>5.0860215053763396</v>
+      </c>
+      <c r="N80" s="6">
+        <f>'By site'!AG12</f>
+        <v>8.4990000000000006</v>
+      </c>
+      <c r="O80" s="5">
+        <f>'By site'!CG12</f>
+        <v>1.1716294458229901E-3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81">
+        <f>'By site'!DN13*'By site'!Z13</f>
+        <v>19.151798216419305</v>
+      </c>
+      <c r="C81" s="5">
+        <f>'By site'!DX13</f>
+        <v>5.4262313508968698E-3</v>
+      </c>
+      <c r="D81" s="2">
+        <f>'By site'!DU13/C81-1</f>
+        <v>0.1819075310481173</v>
+      </c>
+      <c r="E81" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="I81" t="s">
+        <v>83</v>
+      </c>
+      <c r="J81" s="7">
+        <f>'By site'!CD13</f>
+        <v>7265</v>
+      </c>
+      <c r="K81" s="7">
+        <f>'By site'!AD13</f>
+        <v>40</v>
+      </c>
+      <c r="L81">
+        <f>'By site'!AF13</f>
+        <v>33</v>
+      </c>
+      <c r="M81" s="6">
+        <f>'By site'!AQ13</f>
+        <v>5.8016517549896802</v>
+      </c>
+      <c r="N81" s="6">
+        <f>'By site'!AG13</f>
+        <v>8.4909999999999997</v>
+      </c>
+      <c r="O81" s="5">
+        <f>'By site'!CG13</f>
+        <v>1.1687543014452901E-3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
         <v>84</v>
       </c>
-      <c r="B81">
+      <c r="B82">
         <f>'By site'!DN14*'By site'!Z14</f>
         <v>56.321647797862589</v>
       </c>
-      <c r="C81" s="5">
+      <c r="C82" s="5">
         <f>'By site'!DX14</f>
         <v>3.0734467370106002E-3</v>
       </c>
-      <c r="D81" s="2">
-        <f>'By site'!DU14/C81-1</f>
+      <c r="D82" s="2">
+        <f>'By site'!DU14/C82-1</f>
         <v>-0.62383054113809666</v>
       </c>
-      <c r="E81" t="b">
+      <c r="E82" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
+      <c r="I82" t="s">
+        <v>84</v>
+      </c>
+      <c r="J82" s="7">
+        <f>'By site'!CD14</f>
+        <v>12801</v>
+      </c>
+      <c r="K82" s="7">
+        <f>'By site'!AD14</f>
+        <v>64</v>
+      </c>
+      <c r="L82">
+        <f>'By site'!AF14</f>
+        <v>43</v>
+      </c>
+      <c r="M82" s="6">
+        <f>'By site'!AQ14</f>
+        <v>1.72603702835716</v>
+      </c>
+      <c r="N82" s="6">
+        <f>'By site'!AG14</f>
+        <v>29.53</v>
+      </c>
+      <c r="O82" s="5">
+        <f>'By site'!CG14</f>
+        <v>2.3068510272635E-3</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
         <v>72</v>
       </c>
-      <c r="B82">
+      <c r="B83">
         <f>'By site'!DN15*'By site'!Z15</f>
         <v>8.4196860466966505</v>
       </c>
-      <c r="C82" s="5">
+      <c r="C83" s="5">
         <f>'By site'!DX15</f>
         <v>1.8855842445038701E-2</v>
       </c>
-      <c r="D82" s="2">
-        <f>'By site'!DU15/C82-1</f>
+      <c r="D83" s="2">
+        <f>'By site'!DU15/C83-1</f>
         <v>0.67991198879570303</v>
       </c>
-      <c r="E82" t="b">
+      <c r="E83" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
+      <c r="I83" t="s">
+        <v>72</v>
+      </c>
+      <c r="J83" s="7">
+        <f>'By site'!CD15</f>
+        <v>5371</v>
+      </c>
+      <c r="K83" s="7">
+        <f>'By site'!AD15</f>
+        <v>56</v>
+      </c>
+      <c r="L83">
+        <f>'By site'!AF15</f>
+        <v>42</v>
+      </c>
+      <c r="M83" s="6">
+        <f>'By site'!AQ15</f>
+        <v>3.5211320052131798</v>
+      </c>
+      <c r="N83" s="6">
+        <f>'By site'!AG15</f>
+        <v>24.904</v>
+      </c>
+      <c r="O83" s="5">
+        <f>'By site'!CG15</f>
+        <v>4.6367529324148199E-3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
         <v>85</v>
       </c>
-      <c r="B83">
+      <c r="B84">
         <f>'By site'!DN16*'By site'!Z16</f>
         <v>6.9421125078788286</v>
       </c>
-      <c r="C83" s="5">
+      <c r="C84" s="5">
         <f>'By site'!DX16</f>
         <v>5.9587925946185498E-3</v>
       </c>
-      <c r="D83" s="2">
-        <f>'By site'!DU16/C83-1</f>
+      <c r="D84" s="2">
+        <f>'By site'!DU16/C84-1</f>
         <v>-7.4057075467519051E-2</v>
-      </c>
-      <c r="E83" t="b">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>86</v>
-      </c>
-      <c r="B84">
-        <f>'By site'!DN17*'By site'!Z17</f>
-        <v>54.652973052983512</v>
-      </c>
-      <c r="C84" s="5">
-        <f>'By site'!DX17</f>
-        <v>5.9587925946185498E-3</v>
-      </c>
-      <c r="D84" s="2">
-        <f>'By site'!DU17/C84-1</f>
-        <v>3.8283631936311124E-3</v>
       </c>
       <c r="E84" t="b">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="I84" t="s">
+        <v>85</v>
+      </c>
+      <c r="J84" s="7">
+        <f>'By site'!CD16</f>
+        <v>4777</v>
+      </c>
+      <c r="K84" s="7">
+        <f>'By site'!AD16</f>
+        <v>80</v>
+      </c>
+      <c r="L84">
+        <f>'By site'!AF16</f>
+        <v>49</v>
+      </c>
+      <c r="M84" s="6">
+        <f>'By site'!AQ16</f>
+        <v>1.8530458446723901</v>
+      </c>
+      <c r="N84" s="6">
+        <f>'By site'!AG16</f>
+        <v>39.999000000000002</v>
+      </c>
+      <c r="O84" s="5">
+        <f>'By site'!CG16</f>
+        <v>8.3732468076198503E-3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B85">
-        <f>'By site'!DN18*'By site'!Z18</f>
-        <v>41.522548395860255</v>
+        <f>'By site'!DN17*'By site'!Z17</f>
+        <v>54.652973052983512</v>
       </c>
       <c r="C85" s="5">
-        <f>'By site'!DX18</f>
+        <f>'By site'!DX17</f>
         <v>5.9587925946185498E-3</v>
       </c>
       <c r="D85" s="2">
-        <f>'By site'!DU18/C85-1</f>
-        <v>-0.1299571883054208</v>
+        <f>'By site'!DU17/C85-1</f>
+        <v>3.8283631936311124E-3</v>
       </c>
       <c r="E85" t="b">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="I85" t="s">
+        <v>162</v>
+      </c>
+      <c r="J85" s="7">
+        <f>'By site'!CD23</f>
+        <v>104249</v>
+      </c>
+      <c r="K85" s="7"/>
+      <c r="M85" s="6"/>
+      <c r="N85" s="6">
+        <f>'By site'!AG23</f>
+        <v>601.46500000000003</v>
+      </c>
+      <c r="O85" s="3">
+        <f>N85/J85</f>
+        <v>5.7695037842089613E-3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B86">
-        <f>'By site'!DN19*'By site'!Z19</f>
-        <v>13.130424665419572</v>
+        <f>'By site'!DN18*'By site'!Z18</f>
+        <v>41.522548395860255</v>
       </c>
       <c r="C86" s="5">
-        <f>'By site'!DX19</f>
+        <f>'By site'!DX18</f>
         <v>5.9587925946185498E-3</v>
       </c>
       <c r="D86" s="2">
-        <f>'By site'!DU19/C86-1</f>
-        <v>0.42411282020117502</v>
+        <f>'By site'!DU18/C86-1</f>
+        <v>-0.1299571883054208</v>
       </c>
       <c r="E86" t="b">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
+        <v>88</v>
+      </c>
+      <c r="B87">
+        <f>'By site'!DN19*'By site'!Z19</f>
+        <v>13.130424665419572</v>
+      </c>
+      <c r="C87" s="5">
+        <f>'By site'!DX19</f>
+        <v>5.9587925946185498E-3</v>
+      </c>
+      <c r="D87" s="2">
+        <f>'By site'!DU19/C87-1</f>
+        <v>0.42411282020117502</v>
+      </c>
+      <c r="E87" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
         <v>112</v>
       </c>
-      <c r="B87">
+      <c r="B88">
         <f>'By site'!DN20*'By site'!Z20</f>
         <v>28.019992150124839</v>
       </c>
-      <c r="C87" s="5">
+      <c r="C88" s="5">
         <f>'By site'!DX20</f>
         <v>3.0734467370106002E-3</v>
       </c>
-      <c r="D87" s="2">
-        <f>'By site'!DU20/C87-1</f>
+      <c r="D88" s="2">
+        <f>'By site'!DU20/C88-1</f>
         <v>-0.71514678939813114</v>
       </c>
-      <c r="E87" t="b">
+      <c r="E88" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>215</v>
-      </c>
-      <c r="B88">
-        <f>B70+B74+B80+B81+B82+B83</f>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>214</v>
+      </c>
+      <c r="B89">
+        <f>B71+B75+B81+B82+B83+B84</f>
         <v>227.00457410424525</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>216</v>
+      </c>
+      <c r="B90" s="24">
+        <f>B89/'By site'!Z23</f>
+        <v>9.4550194784142547E-3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
         <v>217</v>
       </c>
-      <c r="B89" s="24">
-        <f>B88/'By site'!Z23</f>
-        <v>9.4550194784142547E-3</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
+      <c r="B91">
+        <f>'By site'!S23/B89</f>
+        <v>3.1247810869602906</v>
+      </c>
+    </row>
+    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
         <v>218</v>
       </c>
-      <c r="B90">
-        <f>'By site'!S23/B88</f>
-        <v>3.1247810869602906</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>219</v>
-      </c>
-      <c r="B91">
+      <c r="B92">
         <f>'By site'!BE23/0.0225</f>
         <v>1.3131051574662227</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B94" s="10"/>
     </row>
   </sheetData>
@@ -16441,40 +16908,40 @@
         <v>89</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>232</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>52</v>
@@ -16492,13 +16959,13 @@
         <v>55</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>234</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>235</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>12</v>
@@ -16543,7 +17010,7 @@
         <v>48</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AK1" s="1" t="s">
         <v>16</v>
@@ -16558,7 +17025,7 @@
         <v>119</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AP1" s="1" t="s">
         <v>40</v>
@@ -16576,40 +17043,40 @@
         <v>121</v>
       </c>
       <c r="AU1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="AV1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="BF1" s="1" t="s">
-        <v>248</v>
       </c>
       <c r="BG1" s="1" t="s">
         <v>68</v>
@@ -16720,13 +17187,13 @@
         <v>143</v>
       </c>
       <c r="CQ1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="CR1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="CR1" s="1" t="s">
+      <c r="CS1" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="CS1" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="CT1" s="1" t="s">
         <v>144</v>
@@ -16828,22 +17295,22 @@
         <v>180</v>
       </c>
       <c r="EA1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="EB1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="EB1" s="1" t="s">
+      <c r="EC1" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="EC1" s="1" t="s">
+      <c r="ED1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="ED1" s="1" t="s">
+      <c r="EE1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="EE1" s="1" t="s">
+      <c r="EF1" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="EF1" s="1" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:136" x14ac:dyDescent="0.2">
@@ -17016,7 +17483,7 @@
         <v>28</v>
       </c>
       <c r="AN3" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="AO3" t="s">
         <v>28</v>
@@ -17081,7 +17548,7 @@
       <c r="BI3" s="3">
         <v>1.5772249855008101E-2</v>
       </c>
-      <c r="BJ3">
+      <c r="BJ3" s="3">
         <v>2.9699654238751001E-2</v>
       </c>
       <c r="BK3" s="3">
@@ -18284,40 +18751,40 @@
         <v>89</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>232</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>52</v>
@@ -18335,13 +18802,13 @@
         <v>55</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>234</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>235</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>12</v>
@@ -18386,7 +18853,7 @@
         <v>48</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AK1" s="1" t="s">
         <v>16</v>
@@ -18401,7 +18868,7 @@
         <v>119</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AP1" s="1" t="s">
         <v>40</v>
@@ -18419,40 +18886,40 @@
         <v>121</v>
       </c>
       <c r="AU1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="AV1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="BF1" s="1" t="s">
-        <v>248</v>
       </c>
       <c r="BG1" s="1" t="s">
         <v>68</v>
@@ -18563,13 +19030,13 @@
         <v>143</v>
       </c>
       <c r="CQ1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="CR1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="CR1" s="1" t="s">
+      <c r="CS1" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="CS1" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="CT1" s="1" t="s">
         <v>144</v>
@@ -18671,22 +19138,22 @@
         <v>180</v>
       </c>
       <c r="EA1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="EB1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="EB1" s="1" t="s">
+      <c r="EC1" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="EC1" s="1" t="s">
+      <c r="ED1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="ED1" s="1" t="s">
+      <c r="EE1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="EE1" s="1" t="s">
+      <c r="EF1" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="EF1" s="1" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:136" x14ac:dyDescent="0.2">
@@ -18961,7 +19428,7 @@
         <v>27</v>
       </c>
       <c r="AN5" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="AO5" t="s">
         <v>28</v>

</xml_diff>